<commit_message>
All code received and added. Contribution sheet updated
</commit_message>
<xml_diff>
--- a/CST1500_ContributionSpreadsheet_FINAL_Locked.xlsx
+++ b/CST1500_ContributionSpreadsheet_FINAL_Locked.xlsx
@@ -1,18 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15207BC-E841-4082-8535-2F402EAFB737}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4014B327-829F-4FE5-AE06-1029689A6B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="X4ZlR6JvWvWiB8zDukt5NYZ+6LUTy5vldl3/puEK4WeKo43ORe1O7rqBGokIeM8B6uDTq5MPEFA8n6QMvQb6Ng==" workbookSaltValue="6cw7hsiy8i7NdCSQb2xZ6Q==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group Size 3" sheetId="1" r:id="rId1"/>
     <sheet name="Group Size 2" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -167,20 +180,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -197,19 +206,21 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -230,9 +241,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -270,9 +281,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -305,26 +316,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -357,26 +351,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -554,55 +531,52 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.5703125" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.5546875" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="0.140625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="23.42578125" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="7" max="7" width="17.88671875" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" customWidth="1"/>
+    <col min="9" max="9" width="0.109375" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="23.44140625" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
@@ -635,24 +609,24 @@
       </c>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="2">
         <v>25</v>
       </c>
-      <c r="C8" s="15">
-        <v>0</v>
-      </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="10">
+      <c r="C8" s="11">
+        <v>0</v>
+      </c>
+      <c r="D8" s="12"/>
+      <c r="E8" s="8">
         <v>1</v>
       </c>
-      <c r="F8" s="10">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10">
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
         <v>0</v>
       </c>
       <c r="H8" t="str">
@@ -661,24 +635,24 @@
       </c>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="2">
         <v>25</v>
       </c>
-      <c r="C9" s="15">
-        <v>0</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="10">
+      <c r="C9" s="11">
+        <v>0</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
         <v>1</v>
       </c>
-      <c r="F9" s="10">
-        <v>0</v>
-      </c>
-      <c r="G9" s="10">
+      <c r="G9" s="8">
         <v>0</v>
       </c>
       <c r="H9" t="str">
@@ -687,24 +661,24 @@
       </c>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="2">
         <v>25</v>
       </c>
-      <c r="C10" s="15">
-        <v>0</v>
-      </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="10">
-        <v>0</v>
-      </c>
-      <c r="F10" s="10">
-        <v>0</v>
-      </c>
-      <c r="G10" s="10">
+      <c r="C10" s="11">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12"/>
+      <c r="E10" s="8">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
+        <v>0</v>
+      </c>
+      <c r="G10" s="8">
         <v>1</v>
       </c>
       <c r="H10" t="str">
@@ -713,50 +687,53 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="2">
         <v>15</v>
       </c>
-      <c r="C11" s="15">
-        <v>0</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="F11" s="10">
-        <v>0</v>
-      </c>
-      <c r="G11" s="10">
-        <v>0.5</v>
+      <c r="C11" s="11">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12"/>
+      <c r="E11" s="14">
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F11" s="14">
+        <f>G11</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G11" s="8">
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H11" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(SUM(E11:G11)&lt;&gt;1,IF(SUM(E11:G11)=0, "Not implemented", "Error"),"Ok")</f>
         <v>Ok</v>
       </c>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="2">
         <v>10</v>
       </c>
-      <c r="C12" s="15">
-        <v>0</v>
-      </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="10">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10">
+      <c r="C12" s="11">
+        <v>0</v>
+      </c>
+      <c r="D12" s="12"/>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8">
         <v>0</v>
       </c>
       <c r="H12" t="str">
@@ -764,110 +741,110 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <f>SUM(B8:B12)</f>
         <v>100</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <f>SUM(C8:C12)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="5"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="5">
+      <c r="B14" s="4"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="4">
         <f t="array" ref="E14">SUM(C8:C12*E8:E12)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <f t="array" ref="F14">SUM(C8:C12*F8:F12)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="4">
         <f t="array" ref="G14">SUM(C8:C12*G8:G12)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="4"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <f>AVERAGE(E14,F14,G14)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>B3</f>
         <v>Syed Mohammed Jafer Hussain</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="5">
         <f>IF(E14=0,0,C13  + C13 *(E14-A17)/A17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f>B4</f>
         <v>Amr Asy</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="5">
         <f>IF(F14=0,0,C13  + C13 *(F14-A17)/A17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>B5</f>
         <v>Saifana Maryam</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22" s="5">
         <f>IF(G14=0,0,C13  + C13 *(G14-A17)/A17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="8"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="8"/>
+      <c r="B24" s="6"/>
       <c r="C24" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="str">
         <f>B3</f>
         <v>Syed Mohammed Jafer Hussain</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="9">
         <f>IF(B20&gt;B13,B13, B20)</f>
         <v>0</v>
       </c>
@@ -876,12 +853,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="str">
         <f>B4</f>
         <v>Amr Asy</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="9">
         <f>IF(B21&gt;B13,B13, B21)</f>
         <v>0</v>
       </c>
@@ -890,12 +867,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="str">
         <f>B5</f>
         <v>Saifana Maryam</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="9">
         <f>IF(B22&gt;B13,B13, B22)</f>
         <v>0</v>
       </c>
@@ -904,13 +881,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="17"/>
+    <row r="30" spans="1:3" ht="88.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="13"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
@@ -925,46 +902,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" customWidth="1"/>
+    <col min="1" max="1" width="35.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="4" max="4" width="36.5546875" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="0.140625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="7" max="7" width="0.109375" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="23.44140625" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>16</v>
       </c>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -992,21 +966,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="2">
         <v>25</v>
       </c>
-      <c r="C7" s="15">
-        <v>0</v>
-      </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="10">
-        <v>0</v>
-      </c>
-      <c r="F7" s="10">
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="E7" s="8">
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
         <v>0</v>
       </c>
       <c r="G7" t="str">
@@ -1018,21 +992,21 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="2">
         <v>25</v>
       </c>
-      <c r="C8" s="15">
-        <v>0</v>
-      </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10">
+      <c r="C8" s="11">
+        <v>0</v>
+      </c>
+      <c r="D8" s="12"/>
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
         <v>0</v>
       </c>
       <c r="G8" t="str">
@@ -1044,21 +1018,21 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="2">
         <v>25</v>
       </c>
-      <c r="C9" s="15">
-        <v>0</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="10">
-        <v>0</v>
-      </c>
-      <c r="F9" s="10">
+      <c r="C9" s="11">
+        <v>0</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
         <v>0</v>
       </c>
       <c r="G9" t="str">
@@ -1070,21 +1044,21 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="2">
         <v>15</v>
       </c>
-      <c r="C10" s="15">
-        <v>0</v>
-      </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="10">
-        <v>0</v>
-      </c>
-      <c r="F10" s="10">
+      <c r="C10" s="11">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12"/>
+      <c r="E10" s="8">
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
         <v>0</v>
       </c>
       <c r="G10" t="str">
@@ -1096,21 +1070,21 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="2">
         <v>10</v>
       </c>
-      <c r="C11" s="15">
-        <v>0</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="10">
-        <v>0</v>
-      </c>
-      <c r="F11" s="10">
+      <c r="C11" s="11">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12"/>
+      <c r="E11" s="8">
+        <v>0</v>
+      </c>
+      <c r="F11" s="8">
         <v>0</v>
       </c>
       <c r="G11" t="str">
@@ -1122,90 +1096,90 @@
         <v>Not implemented</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <f>SUM(B7:B11)</f>
         <v>100</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <f>SUM(C7:C11)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="5">
+      <c r="B13" s="4"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="4">
         <f t="array" ref="E13">SUM(C7:C11*E7:E11)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <f t="array" ref="F13">SUM(C7:C11*F7:F11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <f>AVERAGE(E13,F13)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f>B3</f>
         <v>StudentName1</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="5">
         <f>IF(E13=0,0,C12 + C12 *(E13-A16)/A16)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f>B4</f>
         <v>StudentName2</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="5">
         <f>IF(F13=0,0,C12 + C12 *(F13-A16)/A16)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="8"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="8"/>
+      <c r="B22" s="6"/>
       <c r="C22" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="str">
         <f>B3</f>
         <v>StudentName1</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="9">
         <f>IF(B19&gt;B12,B12, B19)</f>
         <v>0</v>
       </c>
@@ -1214,12 +1188,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="str">
         <f>B4</f>
         <v>StudentName2</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="9">
         <f>IF(B20&gt;B12,B12, B20)</f>
         <v>0</v>
       </c>
@@ -1228,13 +1202,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17"/>
+    <row r="27" spans="1:3" ht="109.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="13"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
@@ -1244,6 +1218,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="13086975-c1d0-4a06-9c64-3fd990a1352b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B5E4D76328569F43B69913F006A221B2" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="56a22f8d817eb20ed3693209c2a5d799">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="13086975-c1d0-4a06-9c64-3fd990a1352b" xmlns:ns4="f8d07fca-19e9-492a-8c2e-699b0725e001" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc6f122d176e53dc02b49ce47b3b9659" ns3:_="" ns4:_="">
     <xsd:import namespace="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
@@ -1496,24 +1487,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA851950-2E95-4230-BEB3-A25E4F3EE837}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="f8d07fca-19e9-492a-8c2e-699b0725e001"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="13086975-c1d0-4a06-9c64-3fd990a1352b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCA5D7B-7CC0-427F-B0CE-DC2F534D9F7A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85932C06-FB31-498A-8232-D2B799F2D6AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1530,29 +1529,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCA5D7B-7CC0-427F-B0CE-DC2F534D9F7A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA851950-2E95-4230-BEB3-A25E4F3EE837}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="f8d07fca-19e9-492a-8c2e-699b0725e001"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>